<commit_message>
Bongo BOM . csv
</commit_message>
<xml_diff>
--- a/BongoCay .xlsx
+++ b/BongoCay .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f9a006a4ab87ba7d/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2360448A-81E6-481F-A442-8BD0EBF7BD22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{2360448A-81E6-481F-A442-8BD0EBF7BD22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC107552-56C8-446B-AC54-2AF080257AC4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{766E711F-BBD4-41F6-920B-F79777E7E7D3}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Name</t>
   </si>
@@ -97,6 +97,18 @@
   </si>
   <si>
     <t xml:space="preserve">DigiKey </t>
+  </si>
+  <si>
+    <t>55 MX</t>
+  </si>
+  <si>
+    <t>156 MX</t>
+  </si>
+  <si>
+    <t>93 MX</t>
+  </si>
+  <si>
+    <t>249 MX</t>
   </si>
 </sst>
 </file>
@@ -202,9 +214,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -242,7 +254,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -348,7 +360,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -490,7 +502,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -538,8 +550,8 @@
       <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
+      <c r="D2" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>8</v>
@@ -556,10 +568,10 @@
         <v>11</v>
       </c>
       <c r="C3" s="4">
-        <v>1</v>
-      </c>
-      <c r="D3" s="5">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>12</v>
@@ -578,8 +590,8 @@
       <c r="C4" s="1">
         <v>1</v>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
+      <c r="D4" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>16</v>
@@ -598,8 +610,8 @@
       <c r="C5" s="4">
         <v>1</v>
       </c>
-      <c r="D5" s="5">
-        <v>0</v>
+      <c r="D5" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>19</v>

</xml_diff>